<commit_message>
Perbarui PCB ke revisi TT-PZ2 tanpa ring LED dan IC buffer.
</commit_message>
<xml_diff>
--- a/outputs/01a1753b-8bbf-7951-a911-eb8185920cf5/Checklist-Belanja-TwoTrash.xlsx
+++ b/outputs/01a1753b-8bbf-7951-a911-eb8185920cf5/Checklist-Belanja-TwoTrash.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist belanja" sheetId="1" r:id="R7d79c7a1480b4945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist belanja" sheetId="1" r:id="R85fd942700f94fbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -120,13 +120,13 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="3">
     <x:dxf>
       <x:font>
         <x:color rgb="FF245534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCEEDD"/>
         </x:patternFill>
       </x:fill>
@@ -136,8 +136,18 @@
         <x:color rgb="FF23466B"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF64748B"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDBEAFE"/>
+          <x:bgColor rgb="FFE5E7EB"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -397,7 +407,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>Pi Zero + 2 DRV8825 • PCB TT-PZ1 • Mekanik Rev G1 • 26 Oktober 2026</x:v>
+        <x:v>Pi Zero + 2 DRV8825 • PCB TT-PZ2 • Tanpa WS2812 / IC buffer • 26 Oktober 2026</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -423,7 +433,7 @@
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>Keranjang belum berarti dibeli. Jumlah kosong perlu diukur. Backing plate, Nano dan extension tidak termasuk.</x:v>
+        <x:v>Keranjang belum berarti dibeli. “Tidak perlu” = tidak dibeli untuk TT-PZ2. Jumlah kosong perlu diukur.</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -461,10 +471,11 @@
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="5"/>
       <x:c r="B8" s="5" t="str">
-        <x:v>Jenis barang</x:v>
+        <x:v>Jenis diperlukan</x:v>
       </x:c>
       <x:c r="C8" s="5" t="n">
-        <x:v>64</x:v>
+        <x:f>COUNTIFS(G10:G73,"&lt;&gt;Tidak perlu")</x:f>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
         <x:v>Sudah siap</x:v>
@@ -484,8 +495,8 @@
         <x:v>Belum siap</x:v>
       </x:c>
       <x:c r="I8" s="5" t="n">
-        <x:f>C8-E8-COUNTIFS(G10:G73,"Tidak perlu")</x:f>
-        <x:v>64</x:v>
+        <x:f>C8-E8</x:f>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -635,17 +646,17 @@
         <x:v>SN74AHCT125N, DIP14</x:v>
       </x:c>
       <x:c r="E14" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="2" t="str">
         <x:v>buah</x:v>
       </x:c>
       <x:c r="G14" s="11" t="str">
-        <x:v>Cek stok</x:v>
+        <x:v>Tidak perlu</x:v>
       </x:c>
       <x:c r="H14" s="12" t="str"/>
       <x:c r="I14" s="9" t="str">
-        <x:v>Harus AHCT, bukan 74HC125.</x:v>
+        <x:v>Dihapus pada TT-PZ2: tanpa ring WS2812 dan IC buffer.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -662,16 +673,18 @@
         <x:v>DIP14; lebar 7,62 mm</x:v>
       </x:c>
       <x:c r="E15" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="2" t="str">
         <x:v>buah</x:v>
       </x:c>
       <x:c r="G15" s="11" t="str">
-        <x:v>Cek stok</x:v>
+        <x:v>Tidak perlu</x:v>
       </x:c>
       <x:c r="H15" s="12" t="str"/>
-      <x:c r="I15" s="9" t="str"/>
+      <x:c r="I15" s="9" t="str">
+        <x:v>Dihapus pada TT-PZ2: tanpa ring WS2812 dan IC buffer.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="2" t="n">
@@ -739,7 +752,7 @@
         <x:v>Metal film ¼ W; toleransi 1%</x:v>
       </x:c>
       <x:c r="E18" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F18" s="2" t="str">
         <x:v>buah</x:v>
@@ -864,7 +877,7 @@
         <x:v>Metal film ¼ W; toleransi 1%</x:v>
       </x:c>
       <x:c r="E23" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F23" s="2" t="str">
         <x:v>buah</x:v>
@@ -889,7 +902,7 @@
         <x:v>100 nF / kode 104; pitch 2,54 mm</x:v>
       </x:c>
       <x:c r="E24" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F24" s="2" t="str">
         <x:v>buah</x:v>
@@ -941,17 +954,17 @@
         <x:v>1000 µF 16 V</x:v>
       </x:c>
       <x:c r="E26" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F26" s="2" t="str">
         <x:v>buah</x:v>
       </x:c>
       <x:c r="G26" s="11" t="str">
-        <x:v>Cek stok</x:v>
+        <x:v>Tidak perlu</x:v>
       </x:c>
       <x:c r="H26" s="12" t="str"/>
       <x:c r="I26" s="9" t="str">
-        <x:v>Cocokkan ukuran badan dengan pola PCB.</x:v>
+        <x:v>Dihapus pada TT-PZ2: tanpa ring WS2812 dan IC buffer.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
@@ -1145,16 +1158,18 @@
         <x:v>Pitch 5,08 mm</x:v>
       </x:c>
       <x:c r="E34" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F34" s="2" t="str">
         <x:v>buah</x:v>
       </x:c>
       <x:c r="G34" s="11" t="str">
-        <x:v>Cek stok</x:v>
+        <x:v>Tidak perlu</x:v>
       </x:c>
       <x:c r="H34" s="12" t="str"/>
-      <x:c r="I34" s="9" t="str"/>
+      <x:c r="I34" s="9" t="str">
+        <x:v>Dihapus pada TT-PZ2: tanpa ring WS2812 dan IC buffer.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="48" customHeight="1">
       <x:c r="A35" s="2" t="n">
@@ -1195,7 +1210,7 @@
         <x:v>AWG22 untuk daya/GND; AWG26 untuk sinyal</x:v>
       </x:c>
       <x:c r="E36" s="10" t="n">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F36" s="2" t="str">
         <x:v>potong</x:v>
@@ -1205,7 +1220,7 @@
       </x:c>
       <x:c r="H36" s="12" t="str"/>
       <x:c r="I36" s="9" t="str">
-        <x:v>Panjang sesuai docs/pcb/jumpers.csv; bukan 28 gulung.</x:v>
+        <x:v>22 sambungan W01-W22; panjang mengikuti jumpers.csv TT-PZ2.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
@@ -1296,16 +1311,18 @@
       <x:c r="D40" s="9" t="str">
         <x:v>Tembaga sekitar 0,5 mm²</x:v>
       </x:c>
-      <x:c r="E40" s="10"/>
+      <x:c r="E40" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F40" s="2" t="str">
         <x:v>meter</x:v>
       </x:c>
       <x:c r="G40" s="11" t="str">
-        <x:v>Cek stok</x:v>
+        <x:v>Tidak perlu</x:v>
       </x:c>
       <x:c r="H40" s="12" t="str"/>
       <x:c r="I40" s="9" t="str">
-        <x:v>Ukur kebutuhan panjang pada rakitan.</x:v>
+        <x:v>Dihapus pada TT-PZ2: tanpa ring WS2812 dan IC buffer.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
@@ -1710,7 +1727,9 @@
         <x:v>Cek stok</x:v>
       </x:c>
       <x:c r="H56" s="12" t="str"/>
-      <x:c r="I56" s="9" t="str"/>
+      <x:c r="I56" s="9" t="str">
+        <x:v>TRIG langsung GPIO17 3,3V; ECHO tetap melalui R2/R3. Uji modul yang dibeli.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" s="2" t="n">
@@ -1726,16 +1745,18 @@
         <x:v>WS2812, 12 LED, 5 V</x:v>
       </x:c>
       <x:c r="E57" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F57" s="2" t="str">
         <x:v>buah</x:v>
       </x:c>
       <x:c r="G57" s="11" t="str">
-        <x:v>Cek stok</x:v>
+        <x:v>Tidak perlu</x:v>
       </x:c>
       <x:c r="H57" s="12" t="str"/>
-      <x:c r="I57" s="9" t="str"/>
+      <x:c r="I57" s="9" t="str">
+        <x:v>Dihapus pada TT-PZ2: tanpa ring WS2812 dan IC buffer.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" s="2" t="n">
@@ -2158,6 +2179,9 @@
     </x:cfRule>
     <x:cfRule type="expression" dxfId="1" priority="2">
       <x:formula>G10="Di keranjang"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="2" priority="3">
+      <x:formula>G10="Tidak perlu"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
@@ -2167,7 +2191,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0df0a6daeafc4e64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c09517f81e94fc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>